<commit_message>
Revised Table 1 and S8
</commit_message>
<xml_diff>
--- a/Table_1_S8_Basin Accumulation.xlsx
+++ b/Table_1_S8_Basin Accumulation.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claremurphy-hagan/Desktop/Papers/Sediment Paper/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C093FC56-FDAA-CF4C-A166-62AB70BBFC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD1DE1A-227F-F54B-9CDC-45E68D149FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="1660" windowWidth="24980" windowHeight="17140" xr2:uid="{F2D2D50D-E8C3-D24C-8A19-BBB6293C16CE}"/>
+    <workbookView xWindow="11800" yWindow="1220" windowWidth="23420" windowHeight="17320" xr2:uid="{F2D2D50D-E8C3-D24C-8A19-BBB6293C16CE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table SX" sheetId="1" r:id="rId1"/>
+    <sheet name="Table S8a" sheetId="1" r:id="rId1"/>
+    <sheet name="Table Sb" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="46">
   <si>
     <t>Basin I/III</t>
   </si>
@@ -205,6 +206,21 @@
   <si>
     <t>F</t>
   </si>
+  <si>
+    <t>WY 2021</t>
+  </si>
+  <si>
+    <t>Basin Accumulation (n)</t>
+  </si>
+  <si>
+    <t>Total Fluvial Load (n)</t>
+  </si>
+  <si>
+    <t>Count-based</t>
+  </si>
+  <si>
+    <t>Tons:</t>
+  </si>
 </sst>
 </file>
 
@@ -212,7 +228,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -314,7 +330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -439,12 +455,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -508,39 +539,58 @@
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -889,30 +939,30 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="16"/>
-      <c r="B1" s="40" t="s">
+      <c r="B1" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="40" t="s">
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
-      <c r="J1" s="40" t="s">
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="43" t="s">
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="45"/>
+      <c r="O1" s="54"/>
+      <c r="P1" s="54"/>
+      <c r="Q1" s="55"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="16"/>
@@ -1097,25 +1147,25 @@
       <c r="Q5" s="16"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="38"/>
-      <c r="Q6" s="39"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
+      <c r="M6" s="48"/>
+      <c r="N6" s="48"/>
+      <c r="O6" s="48"/>
+      <c r="P6" s="48"/>
+      <c r="Q6" s="49"/>
     </row>
     <row r="7" spans="1:17" ht="18" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
@@ -1343,25 +1393,25 @@
       <c r="Q11" s="16"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="38"/>
-      <c r="M12" s="38"/>
-      <c r="N12" s="38"/>
-      <c r="O12" s="38"/>
-      <c r="P12" s="38"/>
-      <c r="Q12" s="39"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="48"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="48"/>
+      <c r="M12" s="48"/>
+      <c r="N12" s="48"/>
+      <c r="O12" s="48"/>
+      <c r="P12" s="48"/>
+      <c r="Q12" s="49"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
@@ -1624,25 +1674,25 @@
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38"/>
-      <c r="J17" s="38"/>
-      <c r="K17" s="38"/>
-      <c r="L17" s="38"/>
-      <c r="M17" s="38"/>
-      <c r="N17" s="38"/>
-      <c r="O17" s="38"/>
-      <c r="P17" s="38"/>
-      <c r="Q17" s="39"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="48"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="48"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="48"/>
+      <c r="M17" s="48"/>
+      <c r="N17" s="48"/>
+      <c r="O17" s="48"/>
+      <c r="P17" s="48"/>
+      <c r="Q17" s="49"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
@@ -1756,25 +1806,25 @@
       <c r="Q20" s="25"/>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="38"/>
-      <c r="J21" s="38"/>
-      <c r="K21" s="38"/>
-      <c r="L21" s="38"/>
-      <c r="M21" s="38"/>
-      <c r="N21" s="38"/>
-      <c r="O21" s="38"/>
-      <c r="P21" s="38"/>
-      <c r="Q21" s="39"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="48"/>
+      <c r="L21" s="48"/>
+      <c r="M21" s="48"/>
+      <c r="N21" s="48"/>
+      <c r="O21" s="48"/>
+      <c r="P21" s="48"/>
+      <c r="Q21" s="49"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
@@ -2044,49 +2094,50 @@
         <v>36</v>
       </c>
       <c r="C27" s="35">
-        <v>23000000000</v>
-      </c>
-      <c r="D27" s="35">
-        <v>41000000000</v>
+        <v>23004193416.470699</v>
+      </c>
+      <c r="D27" s="35"/>
+      <c r="E27" s="56" t="s">
+        <v>45</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="G27" s="46">
+      <c r="G27" s="37">
         <f>G22/1000</f>
         <v>1.3214227226199999</v>
       </c>
-      <c r="H27" s="46">
+      <c r="H27" s="37">
         <f t="shared" ref="H27:I27" si="19">H22/1000</f>
         <v>2.7645491405784015</v>
       </c>
-      <c r="I27" s="49">
+      <c r="I27" s="40">
         <f t="shared" si="19"/>
         <v>4.0859718631984014</v>
       </c>
-      <c r="J27" s="47"/>
-      <c r="K27" s="46">
+      <c r="J27" s="38"/>
+      <c r="K27" s="37">
         <f>K22/1000</f>
         <v>1.1406478708524898E-2</v>
       </c>
-      <c r="L27" s="46">
+      <c r="L27" s="37">
         <f t="shared" ref="L27:M27" si="20">L22/1000</f>
         <v>2.5902743425930002E-2</v>
       </c>
-      <c r="M27" s="48">
+      <c r="M27" s="39">
         <f t="shared" si="20"/>
         <v>3.7309222134454902E-2</v>
       </c>
-      <c r="N27" s="47"/>
-      <c r="O27" s="46">
+      <c r="N27" s="38"/>
+      <c r="O27" s="37">
         <f>O22/1000</f>
         <v>3.06986491253442</v>
       </c>
-      <c r="P27" s="46">
+      <c r="P27" s="37">
         <f t="shared" ref="P27:Q27" si="21">P22/1000</f>
         <v>6.1939526085566525</v>
       </c>
-      <c r="Q27" s="49">
+      <c r="Q27" s="40">
         <f t="shared" si="21"/>
         <v>9.263817521091072</v>
       </c>
@@ -2096,49 +2147,47 @@
         <v>37</v>
       </c>
       <c r="C28" s="35">
-        <v>14000000000</v>
-      </c>
-      <c r="D28" s="35">
-        <v>25000000000</v>
-      </c>
+        <v>14971612552.809099</v>
+      </c>
+      <c r="D28" s="35"/>
       <c r="F28" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="G28" s="46">
+      <c r="G28" s="37">
         <f t="shared" ref="G28:I30" si="22">G23/1000</f>
         <v>1.3194418228992002</v>
       </c>
-      <c r="H28" s="46">
+      <c r="H28" s="37">
         <f t="shared" si="22"/>
         <v>2.7619601128448008</v>
       </c>
-      <c r="I28" s="49">
+      <c r="I28" s="40">
         <f t="shared" si="22"/>
         <v>4.081401935744001</v>
       </c>
-      <c r="J28" s="47"/>
-      <c r="K28" s="46">
+      <c r="J28" s="38"/>
+      <c r="K28" s="37">
         <f t="shared" ref="K28:M28" si="23">K23/1000</f>
         <v>1.0823096887502897E-2</v>
       </c>
-      <c r="L28" s="46">
+      <c r="L28" s="37">
         <f t="shared" si="23"/>
         <v>2.5152784367130004E-2</v>
       </c>
-      <c r="M28" s="48">
+      <c r="M28" s="39">
         <f t="shared" si="23"/>
         <v>3.5975881254632899E-2</v>
       </c>
-      <c r="N28" s="47"/>
-      <c r="O28" s="46">
+      <c r="N28" s="38"/>
+      <c r="O28" s="37">
         <f t="shared" ref="O28:Q28" si="24">O23/1000</f>
         <v>3.0665303486818001</v>
       </c>
-      <c r="P28" s="46">
+      <c r="P28" s="37">
         <f t="shared" si="24"/>
         <v>6.1895874293044395</v>
       </c>
-      <c r="Q28" s="49">
+      <c r="Q28" s="40">
         <f t="shared" si="24"/>
         <v>9.2561177779862405</v>
       </c>
@@ -2148,92 +2197,93 @@
         <v>38</v>
       </c>
       <c r="C29" s="35">
-        <v>3900000000</v>
-      </c>
-      <c r="D29" s="35">
-        <v>7000000000</v>
-      </c>
+        <v>4833819594.8614197</v>
+      </c>
+      <c r="D29" s="35"/>
       <c r="F29" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="G29" s="46">
+      <c r="G29" s="37">
         <f t="shared" si="22"/>
         <v>2.3754647908991997E-3</v>
       </c>
-      <c r="H29" s="46">
+      <c r="H29" s="37">
         <f t="shared" si="22"/>
         <v>3.10929403008E-3</v>
       </c>
-      <c r="I29" s="48">
+      <c r="I29" s="39">
         <f t="shared" si="22"/>
         <v>5.4847588209792006E-3</v>
       </c>
-      <c r="J29" s="47"/>
-      <c r="K29" s="46">
+      <c r="J29" s="38"/>
+      <c r="K29" s="37">
         <f t="shared" ref="K29:M30" si="25">K24/1000</f>
         <v>1.9020382930348802E-3</v>
       </c>
-      <c r="L29" s="46">
+      <c r="L29" s="37">
         <f t="shared" si="25"/>
         <v>2.4867243407999998E-3</v>
       </c>
-      <c r="M29" s="48">
+      <c r="M29" s="39">
         <f t="shared" si="25"/>
         <v>4.3887626338348805E-3</v>
       </c>
-      <c r="N29" s="47"/>
-      <c r="O29" s="46">
+      <c r="N29" s="38"/>
+      <c r="O29" s="37">
         <f t="shared" ref="O29:Q30" si="26">O24/1000</f>
         <v>3.5956512953961603E-3</v>
       </c>
-      <c r="P29" s="46">
+      <c r="P29" s="37">
         <f t="shared" si="26"/>
         <v>4.7085079574400003E-3</v>
       </c>
-      <c r="Q29" s="48">
+      <c r="Q29" s="39">
         <f t="shared" si="26"/>
         <v>8.3041592528361619E-3</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>44</v>
+      </c>
       <c r="F30" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="G30" s="46">
+      <c r="G30" s="37">
         <f t="shared" si="22"/>
         <v>0.4310259608054402</v>
       </c>
-      <c r="H30" s="46">
+      <c r="H30" s="37">
         <f t="shared" si="22"/>
         <v>0.68475169647920009</v>
       </c>
-      <c r="I30" s="49">
+      <c r="I30" s="40">
         <f t="shared" si="22"/>
         <v>1.1157776572846403</v>
       </c>
-      <c r="J30" s="47"/>
-      <c r="K30" s="46">
+      <c r="J30" s="38"/>
+      <c r="K30" s="37">
         <f t="shared" si="25"/>
         <v>3.6034732403870196E-3</v>
       </c>
-      <c r="L30" s="46">
+      <c r="L30" s="37">
         <f t="shared" si="25"/>
         <v>5.4360468517599984E-3</v>
       </c>
-      <c r="M30" s="48">
+      <c r="M30" s="39">
         <f t="shared" si="25"/>
         <v>9.039520092147018E-3</v>
       </c>
-      <c r="N30" s="47"/>
-      <c r="O30" s="46">
+      <c r="N30" s="38"/>
+      <c r="O30" s="37">
         <f t="shared" si="26"/>
         <v>0.98877490984672411</v>
       </c>
-      <c r="P30" s="46">
+      <c r="P30" s="37">
         <f t="shared" si="26"/>
         <v>1.4986934616847201</v>
       </c>
-      <c r="Q30" s="49">
+      <c r="Q30" s="40">
         <f t="shared" si="26"/>
         <v>2.4874683715314441</v>
       </c>
@@ -2247,12 +2297,9 @@
       </c>
       <c r="C31" s="36">
         <f>E22/C27</f>
-        <v>0.81295990823424846</v>
-      </c>
-      <c r="D31" s="36">
-        <f>E22/D27</f>
-        <v>0.45605068022896866</v>
-      </c>
+        <v>0.81281171440682365</v>
+      </c>
+      <c r="D31" s="36"/>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
@@ -2263,12 +2310,9 @@
       </c>
       <c r="C32" s="36">
         <f>E23/C28</f>
-        <v>0.83246451467331373</v>
-      </c>
-      <c r="D32" s="36">
-        <f>E23/D28</f>
-        <v>0.46618012821705568</v>
-      </c>
+        <v>0.77844007546399374</v>
+      </c>
+      <c r="D32" s="36"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -2279,12 +2323,9 @@
       </c>
       <c r="C33" s="36">
         <f>E25/C29</f>
-        <v>1.6972904543297924</v>
-      </c>
-      <c r="D33" s="36">
-        <f>E25/D29</f>
-        <v>0.94563325312659863</v>
-      </c>
+        <v>1.3694000452401993</v>
+      </c>
+      <c r="D33" s="36"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C34" s="36"/>
@@ -2303,4 +2344,76 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8290B570-8920-DD45-AFFF-F0B8FCC02E1B}">
+  <dimension ref="A3:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="4" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="45">
+        <v>18698077889.387714</v>
+      </c>
+      <c r="C4" s="45">
+        <v>23004193416.470699</v>
+      </c>
+      <c r="D4" s="46">
+        <f>B4/C4</f>
+        <v>0.81281171440682365</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="45">
+        <v>11654503205.426392</v>
+      </c>
+      <c r="C5" s="45">
+        <v>14971612552.809099</v>
+      </c>
+      <c r="D5" s="46">
+        <f>B5/C5</f>
+        <v>0.77844007546399374</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="45">
+        <v>6619432771.8861904</v>
+      </c>
+      <c r="C6" s="45">
+        <v>4833819594.8614197</v>
+      </c>
+      <c r="D6" s="46">
+        <f>B6/C6</f>
+        <v>1.3694000452401993</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>